<commit_message>
Add raw(ADO用) order xlsx 07/21
</commit_message>
<xml_diff>
--- a/order_0721_raw.xlsx
+++ b/order_0721_raw.xlsx
@@ -607,14 +607,14 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>1632</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>1618</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>1632</t>
-        </is>
-      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>1627</t>
@@ -632,12 +632,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
+          <t>1620</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
           <t>1628</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>1630</t>
         </is>
       </c>
     </row>
@@ -855,37 +855,37 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>4</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>2</t>
         </is>
       </c>
     </row>

</xml_diff>